<commit_message>
saves after final handin
</commit_message>
<xml_diff>
--- a/content/tables/Project2RisksChatGPT.xlsx
+++ b/content/tables/Project2RisksChatGPT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BFH\MSE\MTE7102_DataQualityVisuals\content\tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{834B35EB-5258-423A-8CAE-09374AF2FCED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{690480A5-00E4-4A19-AE4E-DF71D078E486}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" firstSheet="5" activeTab="8" xr2:uid="{C85C79CF-50DE-474C-BA2B-673335091AFF}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" firstSheet="1" activeTab="4" xr2:uid="{C85C79CF-50DE-474C-BA2B-673335091AFF}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -5556,7 +5556,9 @@
       <c r="E4" s="15" t="s">
         <v>359</v>
       </c>
-      <c r="F4" s="16"/>
+      <c r="F4" s="16">
+        <v>20</v>
+      </c>
       <c r="G4" s="16"/>
       <c r="H4" s="16"/>
       <c r="J4" s="19">

</xml_diff>